<commit_message>
RSCD v1.6 — Shaikh (2016) replication bundle: 4 data corrections (S214/S215 12-industry mean, S801 label fix, S1603 T-Bill source, S703 quote), independent-anchor validation architecture, scrubbed docs, repaired CI. See CHANGELOG.md + RELEASE_NOTES.
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extenbooks/S1001_extenbook.xlsx
+++ b/extenbooks/S1001_extenbook.xlsx
@@ -1794,7 +1794,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>**Author**: opus-fanout-ch10</t>
+          <t>**Author**: Anu automated extraction pipeline</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Chapter 10 ("Modern Money and Inflation") opens by arguing that financial-sector profit rates do *not* diverge systematically from industrial profit rates — banking competes for capital like any other industry. Figure 10.1 is the empirical anchor: bank IROP fluctuates around the all-private IROP. Shaikh references Appendix 7.2 (Ch7 industry-level S215 IROP panel) for the underlying derivation.</t>
+          <t>Chapter 10 ("Competition, Finance, and Interest Rates") opens by arguing that financial-sector profit rates do *not* diverge systematically from industrial profit rates — banking competes for capital like any other industry. Figure 10.1 is the empirical anchor: bank IROP fluctuates around the all-private IROP. Shaikh references Appendix 7.2 (Ch7 industry-level S215 IROP panel) for the underlying derivation.</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-18T22:26:02.539593+00:00</t>
+          <t>2026-07-02T06:18:07.676950+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>